<commit_message>
Ajustezs de socios Personal Importacion de Datos
</commit_message>
<xml_diff>
--- a/brio/GruposFamiliares.xlsx
+++ b/brio/GruposFamiliares.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\tsclient\sportivopilar02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{91633599-0258-4A2F-9CCB-CF9AF3130AA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7787E7DE-B5F7-42E1-BDD6-C0E10C281BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13905" xr2:uid="{274503F6-8759-402D-A3CD-B6C588E6D6E3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13905" xr2:uid="{E42EBB0C-78D8-41F4-8F64-8DEA5351E457}"/>
   </bookViews>
   <sheets>
     <sheet name="DATOS SOCIOS" sheetId="1" r:id="rId1"/>
@@ -2946,7 +2946,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1712FE21-E362-40AB-A581-38E1A335BC94}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A223E84C-9AF8-42FA-9156-D017322B5167}">
   <dimension ref="A1:R637"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -10923,7 +10923,7 @@
         <v>220</v>
       </c>
       <c r="L144">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M144" t="s">
         <v>219</v>
@@ -10952,7 +10952,7 @@
         <v>220</v>
       </c>
       <c r="C145">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D145" t="s">
         <v>219</v>
@@ -10979,7 +10979,7 @@
         <v>220</v>
       </c>
       <c r="L145">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M145" t="s">
         <v>219</v>
@@ -11035,7 +11035,7 @@
         <v>220</v>
       </c>
       <c r="L146">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M146" t="s">
         <v>219</v>
@@ -12688,7 +12688,7 @@
         <v>259</v>
       </c>
       <c r="C176">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D176" t="s">
         <v>256</v>
@@ -12912,7 +12912,7 @@
         <v>264</v>
       </c>
       <c r="C180">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D180" t="s">
         <v>261</v>
@@ -16354,7 +16354,7 @@
         <v>343</v>
       </c>
       <c r="C242">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D242" t="s">
         <v>344</v>
@@ -16381,7 +16381,7 @@
         <v>343</v>
       </c>
       <c r="L242">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M242" t="s">
         <v>344</v>
@@ -16437,7 +16437,7 @@
         <v>343</v>
       </c>
       <c r="L243">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M243" t="s">
         <v>344</v>
@@ -16493,7 +16493,7 @@
         <v>343</v>
       </c>
       <c r="L244">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M244" t="s">
         <v>344</v>
@@ -16549,7 +16549,7 @@
         <v>343</v>
       </c>
       <c r="L245">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M245" t="s">
         <v>344</v>
@@ -32536,7 +32536,7 @@
         <v>717</v>
       </c>
       <c r="C533">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D533" t="s">
         <v>718</v>
@@ -32563,7 +32563,7 @@
         <v>717</v>
       </c>
       <c r="L533">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M533" t="s">
         <v>718</v>
@@ -37154,7 +37154,7 @@
         <v>825</v>
       </c>
       <c r="C616">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D616" t="s">
         <v>823</v>

</xml_diff>